<commit_message>
Update Excel sheets and force redownload SHACL
</commit_message>
<xml_diff>
--- a/data/go.xlsx
+++ b/data/go.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11102"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11130"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DE34DDC-5132-F642-91A3-23BB5350E76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F2FF6A68-FBCD-1446-9765-734604BA3C6F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="500" windowWidth="37300" windowHeight="21100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1100" yWindow="500" windowWidth="37300" windowHeight="21100" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Agent" sheetId="18" r:id="rId1"/>
     <sheet name="Doel" sheetId="6" r:id="rId2"/>
-    <sheet name="Leerplan" sheetId="17" r:id="rId3"/>
-    <sheet name="CombLeerdoelOpleidingsniveau" sheetId="19" r:id="rId4"/>
+    <sheet name="DoelCollectie" sheetId="17" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,14 +30,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="232">
   <si>
     <t>CODE</t>
   </si>
   <si>
-    <t>ingerichtDoor</t>
-  </si>
-  <si>
     <t>type</t>
   </si>
   <si>
@@ -555,18 +551,6 @@
     <t>V</t>
   </si>
   <si>
-    <t>leerplan</t>
-  </si>
-  <si>
-    <t>versieDatum</t>
-  </si>
-  <si>
-    <t>collectiedoel</t>
-  </si>
-  <si>
-    <t>collectiedoeltype</t>
-  </si>
-  <si>
     <t>SC-STEM_S-gr2-DoF</t>
   </si>
   <si>
@@ -576,9 +560,6 @@
     <t>Sleutelcompetentie</t>
   </si>
   <si>
-    <t>Competenties inzake wiskunde, exacte wetenschappen en technologie</t>
-  </si>
-  <si>
     <t>06.01</t>
   </si>
   <si>
@@ -739,6 +720,12 @@
   </si>
   <si>
     <t>06.50</t>
+  </si>
+  <si>
+    <t>Leerplan</t>
+  </si>
+  <si>
+    <t>heeftLid</t>
   </si>
 </sst>
 </file>
@@ -836,7 +823,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="14" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -846,6 +832,7 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1196,15 +1183,15 @@
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>123</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>124</v>
       </c>
     </row>
   </sheetData>
@@ -1241,950 +1228,950 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="G1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="7" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="8" t="s">
+        <v>2</v>
+      </c>
+      <c r="K1" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="L1" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="9" t="s">
-        <v>2</v>
-      </c>
-      <c r="I1" s="8" t="s">
+      <c r="M1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="N1" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="O1" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="J1" s="9" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="L1" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="M1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="N1" s="2" t="s">
-        <v>16</v>
-      </c>
-      <c r="O1" s="2" t="s">
-        <v>10</v>
-      </c>
       <c r="P1" s="2" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
     </row>
     <row r="2" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
     </row>
     <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>219</v>
+        <v>213</v>
       </c>
     </row>
     <row r="4" spans="1:16" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>220</v>
+        <v>214</v>
       </c>
     </row>
     <row r="6" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>184</v>
+        <v>178</v>
       </c>
     </row>
     <row r="7" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>221</v>
+        <v>215</v>
       </c>
     </row>
     <row r="8" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>185</v>
+        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
     </row>
     <row r="10" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
     </row>
     <row r="11" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>224</v>
+        <v>218</v>
       </c>
     </row>
     <row r="12" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>225</v>
+        <v>219</v>
       </c>
     </row>
     <row r="13" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>226</v>
+        <v>220</v>
       </c>
     </row>
     <row r="14" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>186</v>
+        <v>180</v>
       </c>
     </row>
     <row r="15" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>227</v>
+        <v>221</v>
       </c>
     </row>
     <row r="16" spans="1:16" ht="64" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>228</v>
+        <v>222</v>
       </c>
     </row>
     <row r="17" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>229</v>
+        <v>223</v>
       </c>
     </row>
     <row r="18" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>187</v>
+        <v>181</v>
       </c>
     </row>
     <row r="19" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>188</v>
+        <v>182</v>
       </c>
     </row>
     <row r="20" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>230</v>
+        <v>224</v>
       </c>
     </row>
     <row r="22" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>231</v>
+        <v>225</v>
       </c>
     </row>
     <row r="23" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>232</v>
+        <v>226</v>
       </c>
     </row>
     <row r="24" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>233</v>
+        <v>227</v>
       </c>
     </row>
     <row r="25" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>190</v>
+        <v>184</v>
       </c>
     </row>
     <row r="26" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
     </row>
     <row r="27" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>193</v>
+        <v>187</v>
       </c>
     </row>
     <row r="28" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>194</v>
+        <v>188</v>
       </c>
     </row>
     <row r="29" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>195</v>
+        <v>189</v>
       </c>
     </row>
     <row r="30" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
     </row>
     <row r="31" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
     </row>
     <row r="32" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
     </row>
     <row r="33" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
     </row>
     <row r="34" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
     </row>
     <row r="35" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>201</v>
+        <v>195</v>
       </c>
     </row>
     <row r="36" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
     </row>
     <row r="37" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
     </row>
     <row r="38" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
     </row>
     <row r="39" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M39" s="1" t="s">
-        <v>205</v>
+        <v>199</v>
       </c>
     </row>
     <row r="40" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M40" s="1" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
     </row>
     <row r="41" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>234</v>
+        <v>228</v>
       </c>
     </row>
     <row r="42" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M42" s="1" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
     </row>
     <row r="43" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M43" s="1" t="s">
-        <v>208</v>
+        <v>202</v>
       </c>
     </row>
     <row r="44" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M44" s="1" t="s">
-        <v>209</v>
+        <v>203</v>
       </c>
     </row>
     <row r="45" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M45" s="1" t="s">
-        <v>210</v>
+        <v>204</v>
       </c>
     </row>
     <row r="46" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M46" s="1" t="s">
-        <v>211</v>
+        <v>205</v>
       </c>
     </row>
     <row r="47" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M47" s="1" t="s">
-        <v>212</v>
+        <v>206</v>
       </c>
     </row>
     <row r="48" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M48" s="1" t="s">
-        <v>213</v>
+        <v>207</v>
       </c>
     </row>
     <row r="49" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M49" s="1" t="s">
-        <v>214</v>
+        <v>208</v>
       </c>
     </row>
     <row r="50" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M50" s="1" t="s">
-        <v>207</v>
+        <v>201</v>
       </c>
     </row>
     <row r="51" spans="1:16" ht="32" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="P51" s="1" t="s">
-        <v>235</v>
+        <v>229</v>
       </c>
     </row>
     <row r="52" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M52" s="1" t="s">
-        <v>215</v>
+        <v>209</v>
       </c>
     </row>
     <row r="53" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M53" s="1" t="s">
-        <v>216</v>
+        <v>210</v>
       </c>
     </row>
     <row r="54" spans="1:16" ht="48" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="M54" s="1" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
     </row>
   </sheetData>
@@ -2196,328 +2183,344 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7618F3A8-AF47-B947-A911-1EFF15E07583}">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:F19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="4" width="40" style="1" customWidth="1"/>
+    <col min="1" max="1" width="40" style="1" customWidth="1"/>
+    <col min="2" max="2" width="68.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" s="2" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" s="2" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="E1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="2" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" ht="16" x14ac:dyDescent="0.2">
+      <c r="F1" s="2" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>140</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>157</v>
+      </c>
+      <c r="E2" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A3" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C3" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D3" s="5" t="s">
         <v>158</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
+      <c r="E3" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
         <v>126</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B4" s="4" t="s">
         <v>142</v>
       </c>
-      <c r="C3" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="C4" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>159</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
+      <c r="E4" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A5" s="5" t="s">
         <v>127</v>
       </c>
-      <c r="B4" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>143</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="C5" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="5" t="s">
         <v>160</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
+      <c r="E5" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>127</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>144</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>160</v>
+      </c>
+      <c r="E6" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A7" s="5" t="s">
         <v>128</v>
       </c>
-      <c r="B5" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="B7" s="5" t="s">
+        <v>145</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>161</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
+      <c r="E7" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
         <v>129</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B8" s="4" t="s">
         <v>146</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="C8" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>162</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
+      <c r="E8" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A9" s="5" t="s">
         <v>130</v>
       </c>
-      <c r="B8" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>147</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="C9" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>163</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
+      <c r="E9" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
         <v>131</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B10" s="4" t="s">
         <v>148</v>
       </c>
-      <c r="C9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="C10" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>164</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+      <c r="E10" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A11" s="5" t="s">
         <v>132</v>
       </c>
-      <c r="B10" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>149</v>
       </c>
-      <c r="C10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="C11" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>165</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
+      <c r="E11" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
         <v>133</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B12" s="4" t="s">
         <v>150</v>
       </c>
-      <c r="C11" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="C12" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D12" s="4" t="s">
         <v>166</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
+      <c r="E12" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="B12" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="C12" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="C13" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D13" s="5" t="s">
         <v>167</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
+      <c r="E13" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
         <v>135</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B14" s="4" t="s">
         <v>152</v>
       </c>
-      <c r="C13" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D13" s="5" t="s">
+      <c r="C14" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>168</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
+      <c r="E14" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A15" s="5" t="s">
         <v>136</v>
       </c>
-      <c r="B14" s="4" t="s">
+      <c r="B15" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="C14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="C15" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
+      <c r="E15" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A16" s="4" t="s">
         <v>137</v>
       </c>
-      <c r="B15" s="5" t="s">
+      <c r="B16" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="C15" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D15" s="5" t="s">
+      <c r="C16" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16" s="4" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
+      <c r="E16" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A17" s="5" t="s">
         <v>138</v>
       </c>
-      <c r="B16" s="4" t="s">
+      <c r="B17" s="5" t="s">
         <v>155</v>
       </c>
-      <c r="C16" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D16" s="4" t="s">
+      <c r="C17" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
+      <c r="E17" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
+      <c r="A18" s="4" t="s">
         <v>139</v>
       </c>
-      <c r="B17" s="5" t="s">
+      <c r="B18" s="4" t="s">
         <v>156</v>
       </c>
-      <c r="C17" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D17" s="5" t="s">
+      <c r="C18" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D18" s="4" t="s">
         <v>172</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
-        <v>140</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>157</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="E18" s="9" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="32" x14ac:dyDescent="0.2">
+      <c r="A19" s="1" t="s">
         <v>173</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2922168E-E57D-9C42-B602-50CC752BD0E2}">
-  <dimension ref="A1:H2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="1" max="8" width="40" style="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:8" s="2" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" s="2" t="s">
+      <c r="B19" s="4" t="s">
         <v>174</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="C19" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="G1" s="2" t="s">
-        <v>176</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>168</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>135</v>
-      </c>
-      <c r="F2" s="6">
-        <v>45688</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>181</v>
+      <c r="F19" s="1" t="s">
+        <v>134</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated changes for webinar
</commit_message>
<xml_diff>
--- a/data/go.xlsx
+++ b/data/go.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="11130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29426"/>
   <workbookPr filterPrivacy="1"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C229D2EE-125D-3743-9348-4840B35F7F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A27536B4-9234-4C99-B9C6-993949477BD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1100" yWindow="500" windowWidth="36900" windowHeight="20700" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Agent" sheetId="18" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="393" uniqueCount="242">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="441" uniqueCount="240">
   <si>
     <t>CODE</t>
   </si>
@@ -402,9 +402,6 @@
     <t>GO!</t>
   </si>
   <si>
-    <t>VOV_SV</t>
-  </si>
-  <si>
     <t>GO_DKO-gr1</t>
   </si>
   <si>
@@ -450,9 +447,6 @@
     <t>GO_V</t>
   </si>
   <si>
-    <t>Leerplannen van het secundair volwassenenonderwijs</t>
-  </si>
-  <si>
     <t>Leerplannen van het deeltijds kunstonderwijs - eerste graad</t>
   </si>
   <si>
@@ -501,9 +495,6 @@
     <t>Opleidingsprofielen van het volwassenenonderwijs</t>
   </si>
   <si>
-    <t>SV</t>
-  </si>
-  <si>
     <t>DKO-gr1</t>
   </si>
   <si>
@@ -757,13 +748,16 @@
   </si>
   <si>
     <t>http://purl.org/dc/terms/Agent</t>
+  </si>
+  <si>
+    <t>isLidVan</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -777,20 +771,6 @@
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri (Body)"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <name val="Calibri (Body)"/>
     </font>
     <font>
       <sz val="8"/>
@@ -814,6 +794,20 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <u/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -829,8 +823,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4" tint="0.79998168889431442"/>
-        <bgColor theme="4" tint="0.79998168889431442"/>
+        <fgColor rgb="FFE0E0E0"/>
+        <bgColor indexed="64"/>
       </patternFill>
     </fill>
   </fills>
@@ -856,39 +850,287 @@
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="31">
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.79998168889431442"/>
+          <bgColor theme="4" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left/>
+        <right/>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE0E0E0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE0E0E0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color auto="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFE0E0E0"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -899,6 +1141,73 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{E47B7121-E182-4F94-82A7-95FC274480AE}" name="Table4" displayName="Table4" ref="A1:B2" totalsRowShown="0" headerRowDxfId="27" dataDxfId="28">
+  <autoFilter ref="A1:B2" xr:uid="{E47B7121-E182-4F94-82A7-95FC274480AE}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{C6D4882D-453E-4891-B2AB-70DE8E86A110}" name="CODE" dataDxfId="30"/>
+    <tableColumn id="2" xr3:uid="{625DE54B-08E1-41DA-8FD6-2B65DF303CCB}" name="naam" dataDxfId="29"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9D39F8FB-FEA4-49FE-8CF0-FCF03C2F5C7F}" name="Table5" displayName="Table5" ref="A1:Q54" totalsRowShown="0" headerRowDxfId="12" dataDxfId="13">
+  <autoFilter ref="A1:Q54" xr:uid="{9D39F8FB-FEA4-49FE-8CF0-FCF03C2F5C7F}"/>
+  <tableColumns count="17">
+    <tableColumn id="1" xr3:uid="{E6F47D15-9CAA-4AB4-87B1-58EDDDB4F813}" name="CODE" dataDxfId="3"/>
+    <tableColumn id="2" xr3:uid="{6BC9552E-6CCB-46A6-ACF6-A1DD922631B1}" name="beschrijving" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{3A9DCE97-B2F3-4949-8B7A-98F243D09DA5}" name="geldigheid" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{62F027C3-3E93-4B34-A2DA-BC6E4967BCD5}" name="identificator" dataDxfId="26"/>
+    <tableColumn id="5" xr3:uid="{A629183C-54FB-4B3B-AE6D-234A9D61FEE7}" name="niveau" dataDxfId="25"/>
+    <tableColumn id="6" xr3:uid="{E0827EC7-7B97-4A36-928D-97DFCAC6B5C4}" name="gedefinieerdDoor" dataDxfId="24"/>
+    <tableColumn id="7" xr3:uid="{BCD00D86-5201-46C3-B6A0-B034789F58F1}" name="onderwerp" dataDxfId="23"/>
+    <tableColumn id="8" xr3:uid="{FE1B3D61-1755-4AA0-A457-01B7913C48FE}" name="type" dataDxfId="22"/>
+    <tableColumn id="9" xr3:uid="{30537236-18AB-451A-95F5-12B865A0F971}" name="bron" dataDxfId="21"/>
+    <tableColumn id="10" xr3:uid="{C507F596-E3EB-4389-9CE9-82C1A6EFD2DA}" name="doelgroep" dataDxfId="20"/>
+    <tableColumn id="11" xr3:uid="{7B998C85-8F1C-40ED-B06C-77BD67E60941}" name="competentie" dataDxfId="19"/>
+    <tableColumn id="12" xr3:uid="{E2140755-FE59-483D-915C-DBB207C2BAFF}" name="gerelateerdAan" dataDxfId="18"/>
+    <tableColumn id="13" xr3:uid="{AD33FB1A-8132-47F1-BF88-24C31C79F140}" name="heeftSpecialisatie" dataDxfId="17"/>
+    <tableColumn id="14" xr3:uid="{A35427BF-47EB-4627-80E3-71F085A231FA}" name="isBrederDan" dataDxfId="16"/>
+    <tableColumn id="15" xr3:uid="{9DC3EDC9-6C80-4326-97A3-0129A12047F8}" name="bestaatUit" dataDxfId="15"/>
+    <tableColumn id="16" xr3:uid="{C609DC05-8241-46B6-92A7-E46D04DCEF4C}" name="gelijkaardig" dataDxfId="14"/>
+    <tableColumn id="17" xr3:uid="{1997A4D3-ABD7-4BD1-878C-1BC65B38E947}" name="isLidVan" dataDxfId="0"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{EF8CE7E8-675A-48E5-864C-349A15463F26}" name="Table3" displayName="Table3" ref="A1:F18" totalsRowShown="0" headerRowDxfId="11">
+  <autoFilter ref="A1:F18" xr:uid="{EF8CE7E8-675A-48E5-864C-349A15463F26}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{C5EA7AA7-4177-48B2-90E4-57D2508D08E8}" name="CODE" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{46330096-A049-4DCA-A0AE-21827919FCDC}" name="naam" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{9C4DE35C-27F5-48D4-B04F-E5B5D6846D87}" name="gedefinieerdDoor" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{64C0B3A2-4D1D-4F11-B08F-F09043119545}" name="niveau" dataDxfId="7"/>
+    <tableColumn id="5" xr3:uid="{15CD021D-1CA0-4C36-9ECC-86744B4BAE8B}" name="type" dataDxfId="6"/>
+    <tableColumn id="6" xr3:uid="{3F218897-9225-4883-84BF-90DA0279CF44}" name="heeftLid" dataDxfId="5"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{A6878FF0-7749-44FC-A66A-D1CEFD6A5627}" name="Table6" displayName="Table6" ref="A1:F2" totalsRowShown="0" headerRowDxfId="4" dataCellStyle="Hyperlink">
+  <autoFilter ref="A1:F2" xr:uid="{A6878FF0-7749-44FC-A66A-D1CEFD6A5627}"/>
+  <tableColumns count="6">
+    <tableColumn id="1" xr3:uid="{15FDDE99-09D8-4A72-BF50-BA900B20A150}" name="sheetLabel"/>
+    <tableColumn id="2" xr3:uid="{0A7441A6-C153-48CD-B5DD-F4D98E6C9D3D}" name="sheetClass" dataCellStyle="Hyperlink"/>
+    <tableColumn id="3" xr3:uid="{B5486C8D-6D7A-4ED5-8005-7F839E553E94}" name="columnLabel"/>
+    <tableColumn id="4" xr3:uid="{1D728D0C-B748-44AA-BB90-D3463AE96DF5}" name="columnProperty" dataCellStyle="Hyperlink"/>
+    <tableColumn id="5" xr3:uid="{CE0704B2-96CD-4811-A431-D841C45FCB4D}" name="valueDatatype" dataCellStyle="Hyperlink"/>
+    <tableColumn id="6" xr3:uid="{D27A4E42-181B-483E-AE48-F094EA2ADF20}" name="valueClass"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight16" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1224,20 +1533,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E48475DD-7AAE-7649-996C-7728C46BB2FB}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="2" width="40" style="1" customWidth="1"/>
+    <col min="1" max="2" width="8.140625" style="1" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:2" s="6" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="16" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>121</v>
       </c>
@@ -1247,88 +1556,95 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:P54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:Q54"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="54.33203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="40" style="1" customWidth="1"/>
-    <col min="5" max="5" width="6.1640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="4.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="4.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="8.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="14.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="10.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="9" style="1" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="9.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="59" style="11" customWidth="1"/>
+    <col min="3" max="3" width="12.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="14.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="7.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8" style="1" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="14.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="17.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="12.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" s="2" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:17" s="7" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="8" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="7" t="s">
         <v>10</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="F1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="G1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="H1" s="7" t="s">
         <v>1</v>
       </c>
       <c r="I1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="8" t="s">
+      <c r="J1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="K1" s="2" t="s">
+      <c r="K1" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="L1" s="2" t="s">
+      <c r="L1" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="M1" s="2" t="s">
-        <v>230</v>
-      </c>
-      <c r="N1" s="2" t="s">
+      <c r="M1" s="7" t="s">
+        <v>227</v>
+      </c>
+      <c r="N1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="O1" s="2" t="s">
+      <c r="O1" s="7" t="s">
         <v>9</v>
       </c>
-      <c r="P1" s="2" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="2" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+      <c r="P1" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="Q1" s="12" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="11" t="s">
         <v>68</v>
       </c>
       <c r="D2" s="1" t="s">
@@ -1338,14 +1654,17 @@
         <v>121</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="3" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+        <v>172</v>
+      </c>
+      <c r="Q2" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="B3" s="1" t="s">
+      <c r="B3" s="11" t="s">
         <v>69</v>
       </c>
       <c r="D3" s="1" t="s">
@@ -1355,14 +1674,17 @@
         <v>121</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="4" spans="1:16" ht="16" x14ac:dyDescent="0.2">
+        <v>208</v>
+      </c>
+      <c r="Q3" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="11" t="s">
         <v>70</v>
       </c>
       <c r="D4" s="1" t="s">
@@ -1372,14 +1694,17 @@
         <v>121</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="5" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>173</v>
+      </c>
+      <c r="Q4" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="11" t="s">
         <v>71</v>
       </c>
       <c r="D5" s="1" t="s">
@@ -1389,14 +1714,17 @@
         <v>121</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>212</v>
-      </c>
-    </row>
-    <row r="6" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>209</v>
+      </c>
+      <c r="Q5" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="11" t="s">
         <v>72</v>
       </c>
       <c r="D6" s="1" t="s">
@@ -1406,14 +1734,17 @@
         <v>121</v>
       </c>
       <c r="M6" s="1" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="7" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>174</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="11" t="s">
         <v>73</v>
       </c>
       <c r="D7" s="1" t="s">
@@ -1423,14 +1754,17 @@
         <v>121</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>213</v>
-      </c>
-    </row>
-    <row r="8" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>210</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="11" t="s">
         <v>74</v>
       </c>
       <c r="D8" s="1" t="s">
@@ -1440,14 +1774,17 @@
         <v>121</v>
       </c>
       <c r="M8" s="1" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="9" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>175</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="11" t="s">
         <v>75</v>
       </c>
       <c r="D9" s="1" t="s">
@@ -1457,14 +1794,17 @@
         <v>121</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="10" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>211</v>
+      </c>
+      <c r="Q9" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="11" t="s">
         <v>76</v>
       </c>
       <c r="D10" s="1" t="s">
@@ -1474,14 +1814,17 @@
         <v>121</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="11" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>212</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="11" t="s">
         <v>77</v>
       </c>
       <c r="D11" s="1" t="s">
@@ -1491,14 +1834,17 @@
         <v>121</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="12" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>213</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="11" t="s">
         <v>78</v>
       </c>
       <c r="D12" s="1" t="s">
@@ -1508,14 +1854,17 @@
         <v>121</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>217</v>
-      </c>
-    </row>
-    <row r="13" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>214</v>
+      </c>
+      <c r="Q12" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="13" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>26</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="11" t="s">
         <v>79</v>
       </c>
       <c r="D13" s="1" t="s">
@@ -1525,14 +1874,17 @@
         <v>121</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>218</v>
-      </c>
-    </row>
-    <row r="14" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>215</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="14" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="11" t="s">
         <v>80</v>
       </c>
       <c r="D14" s="1" t="s">
@@ -1542,14 +1894,17 @@
         <v>121</v>
       </c>
       <c r="M14" s="1" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="15" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>176</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="11" t="s">
         <v>81</v>
       </c>
       <c r="D15" s="1" t="s">
@@ -1559,14 +1914,17 @@
         <v>121</v>
       </c>
       <c r="P15" s="1" t="s">
-        <v>219</v>
-      </c>
-    </row>
-    <row r="16" spans="1:16" ht="64" x14ac:dyDescent="0.2">
+        <v>216</v>
+      </c>
+      <c r="Q15" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="11" t="s">
         <v>82</v>
       </c>
       <c r="D16" s="1" t="s">
@@ -1576,14 +1934,17 @@
         <v>121</v>
       </c>
       <c r="P16" s="1" t="s">
-        <v>220</v>
-      </c>
-    </row>
-    <row r="17" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>217</v>
+      </c>
+      <c r="Q16" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="11" t="s">
         <v>83</v>
       </c>
       <c r="D17" s="1" t="s">
@@ -1593,14 +1954,17 @@
         <v>121</v>
       </c>
       <c r="P17" s="1" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="18" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>218</v>
+      </c>
+      <c r="Q17" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B18" s="1" t="s">
+      <c r="B18" s="11" t="s">
         <v>84</v>
       </c>
       <c r="D18" s="1" t="s">
@@ -1610,14 +1974,17 @@
         <v>121</v>
       </c>
       <c r="M18" s="1" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="19" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>177</v>
+      </c>
+      <c r="Q18" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="19" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B19" s="1" t="s">
+      <c r="B19" s="11" t="s">
         <v>85</v>
       </c>
       <c r="D19" s="1" t="s">
@@ -1627,14 +1994,17 @@
         <v>121</v>
       </c>
       <c r="M19" s="1" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="20" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>178</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B20" s="1" t="s">
+      <c r="B20" s="11" t="s">
         <v>86</v>
       </c>
       <c r="D20" s="1" t="s">
@@ -1644,14 +2014,17 @@
         <v>121</v>
       </c>
       <c r="M20" s="1" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="21" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>179</v>
+      </c>
+      <c r="Q20" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="11" t="s">
         <v>87</v>
       </c>
       <c r="D21" s="1" t="s">
@@ -1661,14 +2034,17 @@
         <v>121</v>
       </c>
       <c r="P21" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="22" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>219</v>
+      </c>
+      <c r="Q21" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="22" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="11" t="s">
         <v>88</v>
       </c>
       <c r="D22" s="1" t="s">
@@ -1678,14 +2054,17 @@
         <v>121</v>
       </c>
       <c r="P22" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="23" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>220</v>
+      </c>
+      <c r="Q22" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="23" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="11" t="s">
         <v>89</v>
       </c>
       <c r="D23" s="1" t="s">
@@ -1695,14 +2074,17 @@
         <v>121</v>
       </c>
       <c r="P23" s="1" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="24" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>221</v>
+      </c>
+      <c r="Q23" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="24" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="B24" s="1" t="s">
+      <c r="B24" s="11" t="s">
         <v>90</v>
       </c>
       <c r="D24" s="1" t="s">
@@ -1712,14 +2094,17 @@
         <v>121</v>
       </c>
       <c r="P24" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="25" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>222</v>
+      </c>
+      <c r="Q24" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="25" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="B25" s="1" t="s">
+      <c r="B25" s="11" t="s">
         <v>91</v>
       </c>
       <c r="D25" s="1" t="s">
@@ -1729,14 +2114,17 @@
         <v>121</v>
       </c>
       <c r="M25" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="26" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>180</v>
+      </c>
+      <c r="Q25" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="26" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="B26" s="1" t="s">
+      <c r="B26" s="11" t="s">
         <v>92</v>
       </c>
       <c r="D26" s="1" t="s">
@@ -1746,14 +2134,17 @@
         <v>121</v>
       </c>
       <c r="M26" s="1" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="27" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>182</v>
+      </c>
+      <c r="Q26" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="27" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="B27" s="1" t="s">
+      <c r="B27" s="11" t="s">
         <v>93</v>
       </c>
       <c r="D27" s="1" t="s">
@@ -1763,14 +2154,17 @@
         <v>121</v>
       </c>
       <c r="M27" s="1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="28" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>183</v>
+      </c>
+      <c r="Q27" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="28" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="B28" s="1" t="s">
+      <c r="B28" s="11" t="s">
         <v>94</v>
       </c>
       <c r="D28" s="1" t="s">
@@ -1780,14 +2174,17 @@
         <v>121</v>
       </c>
       <c r="M28" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="29" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>184</v>
+      </c>
+      <c r="Q28" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="29" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="B29" s="1" t="s">
+      <c r="B29" s="11" t="s">
         <v>95</v>
       </c>
       <c r="D29" s="1" t="s">
@@ -1797,14 +2194,17 @@
         <v>121</v>
       </c>
       <c r="M29" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="30" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>185</v>
+      </c>
+      <c r="Q29" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="30" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="B30" s="1" t="s">
+      <c r="B30" s="11" t="s">
         <v>96</v>
       </c>
       <c r="D30" s="1" t="s">
@@ -1814,14 +2214,17 @@
         <v>121</v>
       </c>
       <c r="M30" s="1" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="31" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>186</v>
+      </c>
+      <c r="Q30" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="31" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="1" t="s">
+      <c r="B31" s="11" t="s">
         <v>97</v>
       </c>
       <c r="D31" s="1" t="s">
@@ -1831,14 +2234,17 @@
         <v>121</v>
       </c>
       <c r="M31" s="1" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="32" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>187</v>
+      </c>
+      <c r="Q31" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="32" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
         <v>45</v>
       </c>
-      <c r="B32" s="1" t="s">
+      <c r="B32" s="11" t="s">
         <v>98</v>
       </c>
       <c r="D32" s="1" t="s">
@@ -1848,14 +2254,17 @@
         <v>121</v>
       </c>
       <c r="M32" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="33" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>188</v>
+      </c>
+      <c r="Q32" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="33" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="B33" s="1" t="s">
+      <c r="B33" s="11" t="s">
         <v>99</v>
       </c>
       <c r="D33" s="1" t="s">
@@ -1865,14 +2274,17 @@
         <v>121</v>
       </c>
       <c r="M33" s="1" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="34" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>189</v>
+      </c>
+      <c r="Q33" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="34" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
         <v>47</v>
       </c>
-      <c r="B34" s="1" t="s">
+      <c r="B34" s="11" t="s">
         <v>100</v>
       </c>
       <c r="D34" s="1" t="s">
@@ -1882,14 +2294,17 @@
         <v>121</v>
       </c>
       <c r="M34" s="1" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="35" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>190</v>
+      </c>
+      <c r="Q34" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="35" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
         <v>48</v>
       </c>
-      <c r="B35" s="1" t="s">
+      <c r="B35" s="11" t="s">
         <v>101</v>
       </c>
       <c r="D35" s="1" t="s">
@@ -1899,14 +2314,17 @@
         <v>121</v>
       </c>
       <c r="M35" s="1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="36" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>191</v>
+      </c>
+      <c r="Q35" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="36" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="B36" s="1" t="s">
+      <c r="B36" s="11" t="s">
         <v>102</v>
       </c>
       <c r="D36" s="1" t="s">
@@ -1916,14 +2334,17 @@
         <v>121</v>
       </c>
       <c r="M36" s="1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="37" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>192</v>
+      </c>
+      <c r="Q36" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="37" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
         <v>50</v>
       </c>
-      <c r="B37" s="1" t="s">
+      <c r="B37" s="11" t="s">
         <v>103</v>
       </c>
       <c r="D37" s="1" t="s">
@@ -1933,14 +2354,17 @@
         <v>121</v>
       </c>
       <c r="M37" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="38" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>193</v>
+      </c>
+      <c r="Q37" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="38" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
         <v>51</v>
       </c>
-      <c r="B38" s="1" t="s">
+      <c r="B38" s="11" t="s">
         <v>104</v>
       </c>
       <c r="D38" s="1" t="s">
@@ -1950,14 +2374,17 @@
         <v>121</v>
       </c>
       <c r="M38" s="1" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="39" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>194</v>
+      </c>
+      <c r="Q38" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="39" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
         <v>52</v>
       </c>
-      <c r="B39" s="1" t="s">
+      <c r="B39" s="11" t="s">
         <v>105</v>
       </c>
       <c r="D39" s="1" t="s">
@@ -1967,14 +2394,17 @@
         <v>121</v>
       </c>
       <c r="N39" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="40" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>195</v>
+      </c>
+      <c r="Q39" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="40" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="B40" s="1" t="s">
+      <c r="B40" s="11" t="s">
         <v>106</v>
       </c>
       <c r="D40" s="1" t="s">
@@ -1984,14 +2414,17 @@
         <v>121</v>
       </c>
       <c r="N40" s="1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="41" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>181</v>
+      </c>
+      <c r="Q40" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="41" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="B41" s="1" t="s">
+      <c r="B41" s="11" t="s">
         <v>107</v>
       </c>
       <c r="D41" s="1" t="s">
@@ -2001,14 +2434,17 @@
         <v>121</v>
       </c>
       <c r="P41" s="1" t="s">
-        <v>226</v>
-      </c>
-    </row>
-    <row r="42" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>223</v>
+      </c>
+      <c r="Q41" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="42" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
         <v>55</v>
       </c>
-      <c r="B42" s="1" t="s">
+      <c r="B42" s="11" t="s">
         <v>108</v>
       </c>
       <c r="D42" s="1" t="s">
@@ -2018,14 +2454,17 @@
         <v>121</v>
       </c>
       <c r="N42" s="1" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="43" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>196</v>
+      </c>
+      <c r="Q42" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="43" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B43" s="1" t="s">
+      <c r="B43" s="11" t="s">
         <v>109</v>
       </c>
       <c r="D43" s="1" t="s">
@@ -2035,14 +2474,17 @@
         <v>121</v>
       </c>
       <c r="N43" s="1" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="44" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>198</v>
+      </c>
+      <c r="Q43" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="44" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
         <v>57</v>
       </c>
-      <c r="B44" s="1" t="s">
+      <c r="B44" s="11" t="s">
         <v>110</v>
       </c>
       <c r="D44" s="1" t="s">
@@ -2052,14 +2494,17 @@
         <v>121</v>
       </c>
       <c r="N44" s="1" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="45" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>199</v>
+      </c>
+      <c r="Q44" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="45" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
         <v>58</v>
       </c>
-      <c r="B45" s="1" t="s">
+      <c r="B45" s="11" t="s">
         <v>111</v>
       </c>
       <c r="D45" s="1" t="s">
@@ -2069,14 +2514,17 @@
         <v>121</v>
       </c>
       <c r="N45" s="1" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="46" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>200</v>
+      </c>
+      <c r="Q45" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="46" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
         <v>59</v>
       </c>
-      <c r="B46" s="1" t="s">
+      <c r="B46" s="11" t="s">
         <v>112</v>
       </c>
       <c r="D46" s="1" t="s">
@@ -2086,14 +2534,17 @@
         <v>121</v>
       </c>
       <c r="N46" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="47" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>201</v>
+      </c>
+      <c r="Q46" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="47" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="B47" s="1" t="s">
+      <c r="B47" s="11" t="s">
         <v>113</v>
       </c>
       <c r="D47" s="1" t="s">
@@ -2103,14 +2554,17 @@
         <v>121</v>
       </c>
       <c r="N47" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="48" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>202</v>
+      </c>
+      <c r="Q47" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="48" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="B48" s="1" t="s">
+      <c r="B48" s="11" t="s">
         <v>114</v>
       </c>
       <c r="D48" s="1" t="s">
@@ -2120,14 +2574,17 @@
         <v>121</v>
       </c>
       <c r="N48" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="49" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>203</v>
+      </c>
+      <c r="Q48" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="49" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="B49" s="1" t="s">
+      <c r="B49" s="11" t="s">
         <v>115</v>
       </c>
       <c r="D49" s="1" t="s">
@@ -2137,14 +2594,17 @@
         <v>121</v>
       </c>
       <c r="N49" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="50" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>204</v>
+      </c>
+      <c r="Q49" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="50" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="B50" s="1" t="s">
+      <c r="B50" s="11" t="s">
         <v>116</v>
       </c>
       <c r="D50" s="1" t="s">
@@ -2154,14 +2614,17 @@
         <v>121</v>
       </c>
       <c r="N50" s="1" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="51" spans="1:16" ht="32" x14ac:dyDescent="0.2">
+        <v>197</v>
+      </c>
+      <c r="Q50" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="51" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A51" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="B51" s="1" t="s">
+      <c r="B51" s="11" t="s">
         <v>117</v>
       </c>
       <c r="D51" s="1" t="s">
@@ -2171,14 +2634,17 @@
         <v>121</v>
       </c>
       <c r="P51" s="1" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="52" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>224</v>
+      </c>
+      <c r="Q51" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="52" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="B52" s="1" t="s">
+      <c r="B52" s="11" t="s">
         <v>118</v>
       </c>
       <c r="D52" s="1" t="s">
@@ -2188,14 +2654,17 @@
         <v>121</v>
       </c>
       <c r="N52" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="53" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>205</v>
+      </c>
+      <c r="Q52" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="53" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="B53" s="1" t="s">
+      <c r="B53" s="11" t="s">
         <v>119</v>
       </c>
       <c r="D53" s="1" t="s">
@@ -2205,14 +2674,17 @@
         <v>121</v>
       </c>
       <c r="N53" s="1" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="54" spans="1:16" ht="48" x14ac:dyDescent="0.2">
+        <v>206</v>
+      </c>
+      <c r="Q53" s="1" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="54" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="B54" s="1" t="s">
+      <c r="B54" s="11" t="s">
         <v>120</v>
       </c>
       <c r="D54" s="1" t="s">
@@ -2222,411 +2694,418 @@
         <v>121</v>
       </c>
       <c r="N54" s="1" t="s">
-        <v>210</v>
+        <v>207</v>
+      </c>
+      <c r="Q54" s="1" t="s">
+        <v>169</v>
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="5" type="noConversion"/>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7618F3A8-AF47-B947-A911-1EFF15E07583}">
-  <dimension ref="A1:F19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:F18"/>
+  <sheetFormatPr defaultColWidth="255.5703125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="40" style="1" customWidth="1"/>
-    <col min="2" max="2" width="68.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="81.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="41.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="2" customFormat="1" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:6" s="9" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="3" t="s">
+      <c r="B1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="7" t="s">
         <v>1</v>
       </c>
-      <c r="F1" s="2" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+      <c r="F1" s="7" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="2" t="s">
+        <v>138</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>154</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F2" s="2"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D2" s="4" t="s">
+      <c r="C3" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>155</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>140</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D4" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="E2" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A3" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="B3" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D3" s="5" t="s">
+      <c r="E4" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F4" s="2"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A5" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>156</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A6" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>142</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D6" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="E3" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A4" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>141</v>
-      </c>
-      <c r="C4" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D4" s="4" t="s">
+      <c r="E6" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" s="2" t="s">
+        <v>127</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>143</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="E4" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A5" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>142</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D5" s="5" t="s">
+      <c r="E7" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A8" s="2" t="s">
+        <v>128</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>144</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D8" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="E5" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A6" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>143</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>159</v>
-      </c>
-      <c r="E6" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A7" s="5" t="s">
-        <v>127</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E8" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A9" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>145</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D9" s="2" t="s">
         <v>160</v>
       </c>
-      <c r="E7" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A8" s="4" t="s">
-        <v>128</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>145</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="E9" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A10" s="2" t="s">
+        <v>130</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="E8" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A9" s="5" t="s">
-        <v>129</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="E10" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F10" s="2"/>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A11" s="2" t="s">
+        <v>131</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>147</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D11" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="E9" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
-        <v>130</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>147</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D10" s="4" t="s">
+      <c r="E11" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A12" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>148</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D12" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="E10" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A11" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="E12" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A13" s="2" t="s">
+        <v>133</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>149</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D13" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="E11" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A12" s="4" t="s">
-        <v>132</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>149</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D12" s="4" t="s">
+      <c r="E13" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>150</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="E12" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A13" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>150</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D13" s="5" t="s">
+      <c r="E14" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A15" s="2" t="s">
+        <v>135</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>151</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D15" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A14" s="4" t="s">
-        <v>134</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>151</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D14" s="4" t="s">
+      <c r="E15" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A16" s="2" t="s">
+        <v>136</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>152</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D16" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="E14" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A15" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="B15" s="5" t="s">
-        <v>152</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D15" s="5" t="s">
+      <c r="E16" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
+        <v>137</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>153</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>168</v>
       </c>
-      <c r="E15" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A16" s="4" t="s">
-        <v>136</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>153</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E16" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A17" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B17" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="2" t="s">
+        <v>225</v>
+      </c>
+      <c r="F17" s="2"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A18" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B18" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="E17" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A18" s="4" t="s">
-        <v>138</v>
-      </c>
-      <c r="B18" s="4" t="s">
-        <v>155</v>
-      </c>
-      <c r="C18" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D18" s="4" t="s">
+      <c r="C18" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="E18" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="E18" s="9" t="s">
-        <v>228</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" ht="16" x14ac:dyDescent="0.2">
-      <c r="A19" s="1" t="s">
-        <v>172</v>
-      </c>
-      <c r="B19" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>121</v>
-      </c>
-      <c r="D19" s="1" t="s">
-        <v>166</v>
-      </c>
-      <c r="E19" s="9" t="s">
-        <v>174</v>
-      </c>
-      <c r="F19" s="1" t="s">
-        <v>133</v>
-      </c>
+      <c r="F18" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2ECD9678-899B-A54F-8349-956CC9BA7BB2}">
   <dimension ref="A1:F2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="39.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="39" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="36.5" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="39.33203125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="29.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="10" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>231</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>232</v>
       </c>
-      <c r="B1" s="10" t="s">
+      <c r="E1" s="3" t="s">
         <v>233</v>
       </c>
-      <c r="C1" s="10" t="s">
+      <c r="F1" s="3" t="s">
         <v>234</v>
       </c>
-      <c r="D1" s="10" t="s">
-        <v>235</v>
-      </c>
-      <c r="E1" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="F1" s="10" t="s">
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" t="s">
-        <v>240</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>241</v>
+      <c r="B2" s="4" t="s">
+        <v>238</v>
       </c>
       <c r="C2" t="s">
         <v>4</v>
       </c>
-      <c r="D2" s="11" t="s">
-        <v>239</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>238</v>
+      <c r="D2" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>235</v>
       </c>
     </row>
   </sheetData>
@@ -2636,5 +3115,8 @@
     <hyperlink ref="E2" r:id="rId3" location="string" xr:uid="{E092415F-AF8C-2247-A460-1D646CC5E6B9}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId4"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>